<commit_message>
Fix export() path bug and align tests with refactored function signatures
- Fix export(): use os.path.join() instead of f-string concatenation
  for output paths, preventing OSError on absolute tmp paths
- Add os.makedirs() for output/ and logs/ folders
- Update test_main.py to match new fetch_page()/scrape_all() signatures
  (config dict as first arg instead of separate search_config)
- Update test_csv_contains_expected_columns to match actual column names
  (Salary Up, Employment Type, Publish Date, Collection date)
- Remove leftover debug print() in scrape_all()
</commit_message>
<xml_diff>
--- a/output/vacancies_result.xlsx
+++ b/output/vacancies_result.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -431,7 +431,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Job Title</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -441,7 +441,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>City</t>
+          <t>Location</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -483,12 +483,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Kierownik / Kierowniczka Robót ds instalacji elektrycznych</t>
+          <t>Kierownik / Kierowniczka Robót Elektrycznych</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>STRABAG</t>
+          <t>TECHBAU BUDOWNICTWO sp. z o.o.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -506,29 +506,29 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-07-16T09:20:48Z</t>
+          <t>2026-07-18T09:22:28Z</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.pl/details/5802404440?utm_medium=api&amp;utm_source=e93aacc2</t>
+          <t>https://www.adzuna.pl/details/5805891424?utm_medium=api&amp;utm_source=e93aacc2</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Kierownik robót elektrycznych (k/m)</t>
+          <t>Kierownik Robót Elektrycznych (k/m/n)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>APER SOLUTION sp. z o.o.</t>
+          <t>Electra M&amp;E Polska Sp. z o.o.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Inżynieria</t>
+          <t>Budownictwo</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -546,29 +546,29 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-07-16T09:20:38Z</t>
+          <t>2026-07-18T09:22:26Z</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://www.adzuna.pl/details/5802403386?utm_medium=api&amp;utm_source=e93aacc2</t>
+          <t>https://www.adzuna.pl/details/5805891269?utm_medium=api&amp;utm_source=e93aacc2</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Kierownik Robót Elektrycznych (k/m/o)</t>
+          <t>Kierownik / Kierowniczka Robót ds instalacji elektrycznych</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SUNHELP ENERGY sp. z o.o.</t>
+          <t>STRABAG</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -586,29 +586,29 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-07-15T21:17:33Z</t>
+          <t>2026-07-16T09:20:48Z</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.pl/details/5801506204?utm_medium=api&amp;utm_source=e93aacc2</t>
+          <t>https://www.adzuna.pl/details/5802404440?utm_medium=api&amp;utm_source=e93aacc2</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Kierownik Robót Elektrycznych</t>
+          <t>Kierownik robót elektrycznych (k/m)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NES Fircroft</t>
+          <t>APER SOLUTION sp. z o.o.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Budownictwo</t>
+          <t>Inżynieria</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
@@ -626,29 +626,29 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-15T09:12:39Z</t>
+          <t>2026-07-16T09:20:38Z</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.pl/details/5800848705?utm_medium=api&amp;utm_source=e93aacc2</t>
+          <t>https://www.adzuna.pl/details/5802403386?utm_medium=api&amp;utm_source=e93aacc2</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Kierownik Robót Elektrycznych M/K</t>
+          <t>Kierownik Robót Elektrycznych (k/m/o)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Grupa KDM sp. z o.o.</t>
+          <t>SUNHELP ENERGY sp. z o.o.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -658,7 +658,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Inżynieria</t>
+          <t>Budownictwo</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
@@ -666,29 +666,29 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-14T17:26:37Z</t>
+          <t>2026-07-15T21:17:33Z</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.pl/details/5800007294?utm_medium=api&amp;utm_source=e93aacc2</t>
+          <t>https://www.adzuna.pl/details/5801506204?utm_medium=api&amp;utm_source=e93aacc2</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Kierownik/czka Robót Elektrycznych</t>
+          <t>Kierownik Robót Elektrycznych</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Climamedic Sp. z o.o. Sp. k.</t>
+          <t>NES Fircroft</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -706,29 +706,29 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-14T09:21:19Z</t>
+          <t>2026-07-15T09:12:39Z</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.pl/details/5799606901?utm_medium=api&amp;utm_source=e93aacc2</t>
+          <t>https://www.adzuna.pl/details/5800848705?utm_medium=api&amp;utm_source=e93aacc2</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Inżynier / Koordynator robót elektrycznych (k/m)</t>
+          <t>Kierownik Robót Elektrycznych M/K</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>REESCO sp. z o.o.</t>
+          <t>Grupa KDM sp. z o.o.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Budownictwo</t>
+          <t>Inżynieria</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
@@ -746,29 +746,29 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-12T12:40:25Z</t>
+          <t>2026-07-14T17:26:37Z</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.pl/details/5797900557?utm_medium=api&amp;utm_source=e93aacc2</t>
+          <t>https://www.adzuna.pl/details/5800007294?utm_medium=api&amp;utm_source=e93aacc2</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Kierownik Robót Elektrycznych (K/M)</t>
+          <t>Kierownik/czka Robót Elektrycznych</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Elemont S.A.</t>
+          <t>Climamedic Sp. z o.o. Sp. k.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -786,29 +786,29 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-12T12:40:20Z</t>
+          <t>2026-07-14T09:21:19Z</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.pl/details/5797899945?utm_medium=api&amp;utm_source=e93aacc2</t>
+          <t>https://www.adzuna.pl/details/5799606901?utm_medium=api&amp;utm_source=e93aacc2</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Asystent kierownika robót elektrycznych</t>
+          <t>Inżynier / Koordynator robót elektrycznych (k/m)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>"Mirmar"s.c. Mirosław Kurczak Marcin Rowicki</t>
+          <t>REESCO sp. z o.o.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -826,29 +826,29 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-12T12:40:17Z</t>
+          <t>2026-07-12T12:40:25Z</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.pl/details/5797899491?utm_medium=api&amp;utm_source=e93aacc2</t>
+          <t>https://www.adzuna.pl/details/5797900557?utm_medium=api&amp;utm_source=e93aacc2</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Kierownik Projektu</t>
+          <t>Kierownik Robót Elektrycznych (K/M)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MICROSYSTEM sp. z o.o.</t>
+          <t>Elemont S.A.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Budownictwo</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -866,29 +866,29 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-11T09:13:49Z</t>
+          <t>2026-07-12T12:40:20Z</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.pl/details/5796630546?utm_medium=api&amp;utm_source=e93aacc2</t>
+          <t>https://www.adzuna.pl/details/5797899945?utm_medium=api&amp;utm_source=e93aacc2</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Inżynier budowy w branży elektrycznej (K/M)</t>
+          <t>Asystent kierownika robót elektrycznych</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Elemont S.A.</t>
+          <t>"Mirmar"s.c. Mirosław Kurczak Marcin Rowicki</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -906,29 +906,29 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-08T10:33:49Z</t>
+          <t>2026-07-12T12:40:17Z</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.pl/details/5792150660?utm_medium=api&amp;utm_source=e93aacc2</t>
+          <t>https://www.adzuna.pl/details/5797899491?utm_medium=api&amp;utm_source=e93aacc2</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Asystent / Asystentka Kierownika Robót Elektrycznych</t>
+          <t>Kierownik Projektu</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>TRZYNERGIA Sp. z o.o.</t>
+          <t>MICROSYSTEM sp. z o.o.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Budownictwo</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -946,29 +946,29 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-08T10:33:10Z</t>
+          <t>2026-07-11T09:13:49Z</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.pl/details/5792150224?utm_medium=api&amp;utm_source=e93aacc2</t>
+          <t>https://www.adzuna.pl/details/5796630546?utm_medium=api&amp;utm_source=e93aacc2</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Inżynier / Kierownik Robót ds. Elektrycznych (K/M/inni)</t>
+          <t>Inżynier budowy w branży elektrycznej (K/M)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>HRK S.A.</t>
+          <t>Elemont S.A.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -986,29 +986,29 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-28T09:10:41Z</t>
+          <t>2026-07-08T10:33:49Z</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.pl/details/5779988813?utm_medium=api&amp;utm_source=e93aacc2</t>
+          <t>https://www.adzuna.pl/details/5792150660?utm_medium=api&amp;utm_source=e93aacc2</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Kierownik Robót Elektrycznych (K/M)</t>
+          <t>Asystent / Asystentka Kierownika Robót Elektrycznych</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BERKER DOMINIS Sp. z o.o. właściciel marki pracownicybudowlani.pl</t>
+          <t>TRZYNERGIA Sp. z o.o.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1026,29 +1026,29 @@
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-28T09:10:39Z</t>
+          <t>2026-07-08T10:33:10Z</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.pl/details/5779988565?utm_medium=api&amp;utm_source=e93aacc2</t>
+          <t>https://www.adzuna.pl/details/5792150224?utm_medium=api&amp;utm_source=e93aacc2</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Kierownik Projektu / Inżynier budowy robót elektrycznych i teletechnicznych (k/m)</t>
+          <t>Inżynier / Kierownik Robót ds. Elektrycznych (K/M/inni)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Quman Sp. o.o.</t>
+          <t>HRK S.A.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1066,29 +1066,29 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-06-27T09:14:06Z</t>
+          <t>2026-06-28T09:10:41Z</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.pl/details/5778823724?utm_medium=api&amp;utm_source=e93aacc2</t>
+          <t>https://www.adzuna.pl/details/5779988813?utm_medium=api&amp;utm_source=e93aacc2</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Kierownik Robót Elektrycznych (k/m/d)</t>
+          <t>Kierownik Robót Elektrycznych (K/M)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ONDE S.A.</t>
+          <t>BERKER DOMINIS Sp. z o.o. właściciel marki pracownicybudowlani.pl</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1106,29 +1106,29 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-06-27T09:07:55Z</t>
+          <t>2026-06-28T09:10:39Z</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.pl/details/5778814987?utm_medium=api&amp;utm_source=e93aacc2</t>
+          <t>https://www.adzuna.pl/details/5779988565?utm_medium=api&amp;utm_source=e93aacc2</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Kierownik robót elektrycznych i teletechnicznych</t>
+          <t>Kierownik Robót Elektrycznych (k/m/d)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ADW Projekt Sp. z o. o.</t>
+          <t>ONDE S.A.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1146,29 +1146,29 @@
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-06-26T09:02:14Z</t>
+          <t>2026-06-27T09:07:55Z</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.pl/details/5777376000?utm_medium=api&amp;utm_source=e93aacc2</t>
+          <t>https://www.adzuna.pl/details/5778814987?utm_medium=api&amp;utm_source=e93aacc2</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Kierownik robót branży elektrycznej (k/m)</t>
+          <t>Kierownik robót elektrycznych i teletechnicznych</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Control Process SA</t>
+          <t>ADW Projekt Sp. z o. o.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1186,29 +1186,29 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-06-26T09:02:12Z</t>
+          <t>2026-06-26T09:02:14Z</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.pl/details/5777375697?utm_medium=api&amp;utm_source=e93aacc2</t>
+          <t>https://www.adzuna.pl/details/5777376000?utm_medium=api&amp;utm_source=e93aacc2</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Kierownik / Kierowniczka robót elektrycznych na projekcie kubaturowym</t>
+          <t>Kierownik robót branży elektrycznej (k/m)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>MIRBUD S.A.</t>
+          <t>Control Process SA</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Budownictwo</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
@@ -1226,177 +1226,17 @@
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-06-19T15:52:33Z</t>
+          <t>2026-06-26T09:02:12Z</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.pl/details/5769403058?utm_medium=api&amp;utm_source=e93aacc2</t>
+          <t>https://www.adzuna.pl/details/5777375697?utm_medium=api&amp;utm_source=e93aacc2</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Kierownik / Kierowniczka robót elektrycznych na projekcie kubaturowym</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>MIRBUD S.A.</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Warszawa, mazowieckie</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Budownictwo</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>2026-06-19T08:55:12Z</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.pl/details/5769099389?utm_medium=api&amp;utm_source=e93aacc2</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Kierownik / Kierowniczka Robót Elektrycznych</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Chemobudowa</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Warszawa, mazowieckie</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Budownictwo</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>2026-06-19T08:55:05Z</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.pl/details/5769098783?utm_medium=api&amp;utm_source=e93aacc2</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Kierownik / Kierowniczka robót elektrycznych</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Euroklimat sp. z o.o.</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Warszawa, mazowieckie</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Budownictwo</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>2026-06-17T21:05:03Z</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.pl/details/5766981309?utm_medium=api&amp;utm_source=e93aacc2</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Kierownik projektu/robót elektrycznych (m/k)</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>BLAKS Spółka Akcyjna</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Warszawa, mazowieckie</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Budownictwo</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>2026-06-17T21:04:07Z</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.pl/details/5766979055?utm_medium=api&amp;utm_source=e93aacc2</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>

</xml_diff>